<commit_message>
Add 4 participants (Erling, Kari SJ, Liza, Mari BH); use filename verbatim as display name
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Toppscorar alle.xlsx
+++ b/Toppscorar alle.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uio.sharepoint.com/sites/VM-tippekonk/Delte dokumenter/General/Innsendte skjema/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="42" documentId="8_{3B660BEF-3346-45CC-A4AD-6AFEA43A43DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{054F26F4-189F-4CD4-9FA2-7632DD90B463}"/>
+  <xr:revisionPtr revIDLastSave="50" documentId="8_{3B660BEF-3346-45CC-A4AD-6AFEA43A43DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{93B2C485-2CC6-4149-8871-58DC91999C2C}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{E70A061D-18D6-4C5B-80EF-E3D3B5B86806}"/>
+    <workbookView xWindow="7410" yWindow="1770" windowWidth="26280" windowHeight="17775" xr2:uid="{E70A061D-18D6-4C5B-80EF-E3D3B5B86806}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="37">
   <si>
     <t>Toppscorar</t>
   </si>
@@ -135,13 +135,28 @@
   </si>
   <si>
     <t>Nina</t>
+  </si>
+  <si>
+    <t>Erling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oyarzabal </t>
+  </si>
+  <si>
+    <t>Kari SJ</t>
+  </si>
+  <si>
+    <t>Liza</t>
+  </si>
+  <si>
+    <t>Mari BH</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -176,6 +191,13 @@
       <family val="2"/>
       <scheme val="major"/>
     </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF000014"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -197,7 +219,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -206,6 +228,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -223,12 +246,8 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office-tema">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -544,171 +563,194 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52A86B2F-151B-4EF3-B3A3-8AA4CF37498E}">
-  <dimension ref="A1:B22"/>
-  <sheetFormatPr defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:B25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.453125" style="4" customWidth="1"/>
-    <col min="2" max="2" width="28.453125" style="4" customWidth="1"/>
-    <col min="3" max="16384" width="11.453125" style="4"/>
+    <col min="1" max="1" width="23.42578125" style="4" customWidth="1"/>
+    <col min="2" max="2" width="28.42578125" style="4" customWidth="1"/>
+    <col min="3" max="16384" width="11.42578125" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A6" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B8" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A9" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A10" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A11" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A12" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A13" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B15" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A16" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="16" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+        <v>26</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+        <v>28</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="4" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -717,21 +759,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x01010090E39FCCE5B25D41843728463D8702CD" ma:contentTypeVersion="3" ma:contentTypeDescription="Opprett et nytt dokument." ma:contentTypeScope="" ma:versionID="f526c9bbb9da171fc3aa15898664257d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3dacec4a-16e0-4c23-af47-b0328532aa0c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9f692aa5e1eb72d1d7d7719d109e8ca1" ns2:_="">
     <xsd:import namespace="3dacec4a-16e0-4c23-af47-b0328532aa0c"/>
@@ -869,15 +902,16 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF27B022-6D43-4647-B8FD-7B1F7A621ED1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AED54E6B-1D4D-40A6-8E6D-B0E7E16AEBF0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -893,7 +927,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A262A202-3D81-4029-A6DD-891A659C9135}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -909,4 +943,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF27B022-6D43-4647-B8FD-7B1F7A621ED1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>